<commit_message>
Pixel Border test (Modify)
Pixelated border variant for the Modifier cards
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concepts/Cards by Layer.xlsx
+++ b/Assets/Documents/Concepts/Cards by Layer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\Cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB32419F-7CCE-4B71-A28D-D6C1FBFFF560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8E494A-AFA7-47A2-8BC1-811D6443AA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attack" sheetId="10" r:id="rId1"/>
@@ -253,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -504,6 +504,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -17126,6 +17129,13 @@
             <a:schemeClr val="tx1"/>
           </a:solidFill>
         </a:ln>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT prst="angle"/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -17197,6 +17207,13 @@
             <a:schemeClr val="tx1"/>
           </a:solidFill>
         </a:ln>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT prst="angle"/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -17268,6 +17285,13 @@
             <a:schemeClr val="tx1"/>
           </a:solidFill>
         </a:ln>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT prst="angle"/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -17340,6 +17364,13 @@
           </a:solidFill>
         </a:ln>
         <a:effectLst/>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT w="152400" h="50800" prst="softRound"/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -17412,6 +17443,13 @@
           </a:solidFill>
         </a:ln>
         <a:effectLst/>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT w="152400" h="50800" prst="softRound"/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -19477,6 +19515,13 @@
           </a:solidFill>
         </a:ln>
         <a:effectLst/>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT w="165100" prst="coolSlant"/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="3">
@@ -19505,13 +19550,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
+      <xdr:col>25</xdr:col>
       <xdr:colOff>95248</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>109849</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>26</xdr:col>
       <xdr:colOff>798206</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>366740</xdr:rowOff>
@@ -19529,7 +19574,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="15667757" y="414649"/>
+          <a:off x="21680630" y="414649"/>
           <a:ext cx="1090885" cy="1088164"/>
           <a:chOff x="7552765" y="1580029"/>
           <a:chExt cx="720000" cy="720000"/>
@@ -19786,13 +19831,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>179554</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>109849</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>357407</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>409978</xdr:rowOff>
@@ -19810,7 +19855,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20282499" y="414649"/>
+          <a:off x="26295372" y="414649"/>
           <a:ext cx="1549453" cy="1131402"/>
           <a:chOff x="7021203" y="1580029"/>
           <a:chExt cx="438150" cy="330299"/>
@@ -20083,6 +20128,13 @@
             <a:schemeClr val="tx1"/>
           </a:solidFill>
         </a:ln>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="threePt" dir="t"/>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT/>
+        </a:sp3d>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="2">
@@ -20113,6 +20165,56 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>27710</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>3001</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{126394C9-BCE5-FC1E-BDE5-3A7FFD3821B1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14159345" y="304800"/>
+          <a:ext cx="5818910" cy="7858528"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -20430,11 +20532,11 @@
       <c r="M3" s="64"/>
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
-      <c r="R3" s="122"/>
-      <c r="S3" s="122"/>
-      <c r="T3" s="122"/>
-      <c r="U3" s="122"/>
-      <c r="V3" s="122"/>
+      <c r="R3" s="123"/>
+      <c r="S3" s="123"/>
+      <c r="T3" s="123"/>
+      <c r="U3" s="123"/>
+      <c r="V3" s="123"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="2"/>
       <c r="AB3" s="64"/>
@@ -20452,11 +20554,11 @@
       <c r="M4" s="65"/>
       <c r="N4" s="63"/>
       <c r="O4" s="5"/>
-      <c r="R4" s="122"/>
-      <c r="S4" s="122"/>
-      <c r="T4" s="122"/>
-      <c r="U4" s="122"/>
-      <c r="V4" s="122"/>
+      <c r="R4" s="123"/>
+      <c r="S4" s="123"/>
+      <c r="T4" s="123"/>
+      <c r="U4" s="123"/>
+      <c r="V4" s="123"/>
       <c r="Z4" s="4"/>
       <c r="AA4" s="63"/>
       <c r="AB4" s="65"/>
@@ -20474,11 +20576,11 @@
       <c r="M5" s="66"/>
       <c r="N5" s="63"/>
       <c r="O5" s="5"/>
-      <c r="R5" s="122"/>
-      <c r="S5" s="122"/>
-      <c r="T5" s="122"/>
-      <c r="U5" s="122"/>
-      <c r="V5" s="122"/>
+      <c r="R5" s="123"/>
+      <c r="S5" s="123"/>
+      <c r="T5" s="123"/>
+      <c r="U5" s="123"/>
+      <c r="V5" s="123"/>
       <c r="Z5" s="4"/>
       <c r="AA5" s="63"/>
       <c r="AB5" s="65"/>
@@ -20496,11 +20598,11 @@
       <c r="M6" s="60"/>
       <c r="N6" s="61"/>
       <c r="O6" s="5"/>
-      <c r="R6" s="122"/>
-      <c r="S6" s="122"/>
-      <c r="T6" s="122"/>
-      <c r="U6" s="122"/>
-      <c r="V6" s="122"/>
+      <c r="R6" s="123"/>
+      <c r="S6" s="123"/>
+      <c r="T6" s="123"/>
+      <c r="U6" s="123"/>
+      <c r="V6" s="123"/>
       <c r="Z6" s="4"/>
       <c r="AA6" s="78"/>
       <c r="AB6" s="78"/>
@@ -20518,11 +20620,11 @@
       <c r="M7" s="74"/>
       <c r="N7" s="74"/>
       <c r="O7" s="75"/>
-      <c r="R7" s="122"/>
-      <c r="S7" s="122"/>
-      <c r="T7" s="122"/>
-      <c r="U7" s="122"/>
-      <c r="V7" s="122"/>
+      <c r="R7" s="123"/>
+      <c r="S7" s="123"/>
+      <c r="T7" s="123"/>
+      <c r="U7" s="123"/>
+      <c r="V7" s="123"/>
       <c r="Z7" s="4"/>
       <c r="AA7" s="74"/>
       <c r="AB7" s="74"/>
@@ -20540,11 +20642,11 @@
       <c r="M8" s="72"/>
       <c r="N8" s="72"/>
       <c r="O8" s="7"/>
-      <c r="R8" s="122"/>
-      <c r="S8" s="122"/>
-      <c r="T8" s="122"/>
-      <c r="U8" s="122"/>
-      <c r="V8" s="122"/>
+      <c r="R8" s="123"/>
+      <c r="S8" s="123"/>
+      <c r="T8" s="123"/>
+      <c r="U8" s="123"/>
+      <c r="V8" s="123"/>
       <c r="Z8" s="6"/>
       <c r="AA8" s="72"/>
       <c r="AB8" s="72"/>
@@ -21375,7 +21477,7 @@
   <sheetPr>
     <tabColor theme="3" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="C2:W9"/>
+  <dimension ref="C2:AD9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="1.6640625" customWidth="1"/>
@@ -21392,19 +21494,25 @@
     <col min="13" max="13" width="47.6640625" customWidth="1"/>
     <col min="14" max="14" width="12.6640625" customWidth="1"/>
     <col min="15" max="15" width="5.6640625" customWidth="1"/>
-    <col min="16" max="16" width="1.6640625" customWidth="1"/>
-    <col min="17" max="17" width="20.6640625" customWidth="1"/>
-    <col min="18" max="18" width="1.6640625" customWidth="1"/>
-    <col min="19" max="19" width="5.6640625" customWidth="1"/>
-    <col min="20" max="20" width="12.6640625" customWidth="1"/>
-    <col min="21" max="21" width="47.6640625" customWidth="1"/>
-    <col min="22" max="22" width="12.6640625" customWidth="1"/>
-    <col min="23" max="23" width="5.6640625" customWidth="1"/>
-    <col min="24" max="24" width="1.6640625" customWidth="1"/>
+    <col min="16" max="17" width="1.6640625" customWidth="1"/>
+    <col min="18" max="18" width="5.6640625" customWidth="1"/>
+    <col min="19" max="19" width="12.6640625" customWidth="1"/>
+    <col min="20" max="20" width="47.6640625" customWidth="1"/>
+    <col min="21" max="21" width="12.6640625" customWidth="1"/>
+    <col min="22" max="22" width="5.6640625" customWidth="1"/>
+    <col min="23" max="23" width="1.6640625" customWidth="1"/>
+    <col min="24" max="24" width="20.6640625" customWidth="1"/>
+    <col min="25" max="25" width="1.6640625" customWidth="1"/>
+    <col min="26" max="26" width="5.6640625" customWidth="1"/>
+    <col min="27" max="27" width="12.6640625" customWidth="1"/>
+    <col min="28" max="28" width="47.6640625" customWidth="1"/>
+    <col min="29" max="29" width="12.6640625" customWidth="1"/>
+    <col min="30" max="30" width="5.6640625" customWidth="1"/>
+    <col min="31" max="31" width="1.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:23" ht="10.050000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="3:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:30" ht="10.050000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="3:30" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C3" s="30"/>
       <c r="D3" s="31"/>
       <c r="E3" s="116"/>
@@ -21415,13 +21523,18 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="3"/>
+      <c r="R3" s="122"/>
+      <c r="S3" s="122"/>
+      <c r="T3" s="122"/>
+      <c r="U3" s="122"/>
+      <c r="V3" s="122"/>
+      <c r="Z3" s="1"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="3"/>
     </row>
-    <row r="4" spans="3:23" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:30" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C4" s="33"/>
       <c r="D4" s="120"/>
       <c r="E4" s="117"/>
@@ -21432,13 +21545,18 @@
       <c r="M4" s="8"/>
       <c r="N4" s="63"/>
       <c r="O4" s="5"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="63"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="63"/>
-      <c r="W4" s="5"/>
+      <c r="R4" s="122"/>
+      <c r="S4" s="122"/>
+      <c r="T4" s="122"/>
+      <c r="U4" s="122"/>
+      <c r="V4" s="122"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="63"/>
+      <c r="AB4" s="65"/>
+      <c r="AC4" s="63"/>
+      <c r="AD4" s="5"/>
     </row>
-    <row r="5" spans="3:23" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:30" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C5" s="33"/>
       <c r="D5" s="120"/>
       <c r="E5" s="117"/>
@@ -21449,13 +21567,18 @@
       <c r="M5" s="8"/>
       <c r="N5" s="63"/>
       <c r="O5" s="5"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="63"/>
-      <c r="U5" s="65"/>
-      <c r="V5" s="63"/>
-      <c r="W5" s="5"/>
+      <c r="R5" s="122"/>
+      <c r="S5" s="122"/>
+      <c r="T5" s="122"/>
+      <c r="U5" s="122"/>
+      <c r="V5" s="122"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="63"/>
+      <c r="AB5" s="65"/>
+      <c r="AC5" s="63"/>
+      <c r="AD5" s="5"/>
     </row>
-    <row r="6" spans="3:23" ht="288" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="3:30" ht="288" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C6" s="33"/>
       <c r="D6" s="121"/>
       <c r="E6" s="121"/>
@@ -21466,13 +21589,18 @@
       <c r="M6" s="112"/>
       <c r="N6" s="113"/>
       <c r="O6" s="5"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="78"/>
-      <c r="U6" s="78"/>
-      <c r="V6" s="78"/>
-      <c r="W6" s="5"/>
+      <c r="R6" s="122"/>
+      <c r="S6" s="122"/>
+      <c r="T6" s="122"/>
+      <c r="U6" s="122"/>
+      <c r="V6" s="122"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="78"/>
+      <c r="AB6" s="78"/>
+      <c r="AC6" s="78"/>
+      <c r="AD6" s="5"/>
     </row>
-    <row r="7" spans="3:23" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:30" ht="169.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="33"/>
       <c r="D7" s="118"/>
       <c r="E7" s="118"/>
@@ -21483,13 +21611,18 @@
       <c r="M7" s="114"/>
       <c r="N7" s="114"/>
       <c r="O7" s="5"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="74"/>
-      <c r="U7" s="74"/>
-      <c r="V7" s="74"/>
-      <c r="W7" s="75"/>
+      <c r="R7" s="122"/>
+      <c r="S7" s="122"/>
+      <c r="T7" s="122"/>
+      <c r="U7" s="122"/>
+      <c r="V7" s="122"/>
+      <c r="Z7" s="4"/>
+      <c r="AA7" s="74"/>
+      <c r="AB7" s="74"/>
+      <c r="AC7" s="74"/>
+      <c r="AD7" s="75"/>
     </row>
-    <row r="8" spans="3:23" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:30" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C8" s="35"/>
       <c r="D8" s="115"/>
       <c r="E8" s="115"/>
@@ -21500,27 +21633,33 @@
       <c r="M8" s="72"/>
       <c r="N8" s="72"/>
       <c r="O8" s="7"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="72"/>
-      <c r="U8" s="72"/>
-      <c r="V8" s="72"/>
-      <c r="W8" s="7"/>
+      <c r="R8" s="122"/>
+      <c r="S8" s="122"/>
+      <c r="T8" s="122"/>
+      <c r="U8" s="122"/>
+      <c r="V8" s="122"/>
+      <c r="Z8" s="6"/>
+      <c r="AA8" s="72"/>
+      <c r="AB8" s="72"/>
+      <c r="AC8" s="72"/>
+      <c r="AD8" s="7"/>
     </row>
-    <row r="9" spans="3:23" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="3:30" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="T8:V8"/>
+  <mergeCells count="18">
+    <mergeCell ref="AA8:AC8"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="E3:E5"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="D6:F6"/>
-    <mergeCell ref="U3:U5"/>
-    <mergeCell ref="T4:T5"/>
-    <mergeCell ref="V4:V5"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="R3:V8"/>
+    <mergeCell ref="AB3:AB5"/>
+    <mergeCell ref="AA4:AA5"/>
+    <mergeCell ref="AC4:AC5"/>
+    <mergeCell ref="AA6:AC6"/>
+    <mergeCell ref="AA7:AD7"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="N4:N5"/>
     <mergeCell ref="L6:N6"/>

</xml_diff>